<commit_message>
feat: add some fields on invoice-mtt crud and import
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoice_mtt/MauUploadHDMTT-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoice_mtt/MauUploadHDMTT-TT78.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="23040" windowHeight="8940"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,12 +30,25 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
+    <author>trann</author>
     <author>haof</author>
     <author>ASIA</author>
     <author>nguyen hungn</author>
   </authors>
   <commentList>
-    <comment ref="K1" authorId="0">
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Cách nhau bơi dấu ,</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -50,7 +63,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="1">
+    <comment ref="O1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -68,7 +81,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="1">
+    <comment ref="V1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -90,7 +103,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0">
+    <comment ref="X1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -112,7 +125,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="1">
+    <comment ref="Y1" authorId="2">
       <text>
         <r>
           <rPr>
@@ -137,7 +150,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="2">
+    <comment ref="AA1" authorId="3">
       <text>
         <r>
           <rPr>
@@ -155,7 +168,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
   <si>
     <t>MaHD(*)</t>
   </si>
@@ -166,9 +179,15 @@
     <t>TenNguoiMua</t>
   </si>
   <si>
+    <t>MaSoDVQHNS</t>
+  </si>
+  <si>
     <t>CCCD</t>
   </si>
   <si>
+    <t>SoHoChieu</t>
+  </si>
+  <si>
     <t>TenDonVi</t>
   </si>
   <si>
@@ -176,6 +195,9 @@
   </si>
   <si>
     <t>MailKhachHang</t>
+  </si>
+  <si>
+    <t>MailCC</t>
   </si>
   <si>
     <t>SoDienThoaiKH</t>
@@ -335,7 +357,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,11 +516,6 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
@@ -507,6 +524,21 @@
       <charset val="0"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
@@ -514,11 +546,6 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
@@ -999,10 +1026,10 @@
     <xf numFmtId="1" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1327,31 +1354,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Y9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <dimension ref="A1:AB6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
     <col min="2" max="2" width="11.8190476190476" style="2" customWidth="1"/>
-    <col min="3" max="3" width="16" style="2" customWidth="1"/>
-    <col min="4" max="5" width="12.7238095238095" customWidth="1"/>
-    <col min="6" max="7" width="19.1809523809524" customWidth="1"/>
-    <col min="8" max="8" width="15.2666666666667" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="12.8190476190476" customWidth="1"/>
-    <col min="11" max="12" width="22.1809523809524" style="3" customWidth="1"/>
-    <col min="13" max="13" width="11.5428571428571" customWidth="1"/>
-    <col min="14" max="14" width="15.447619047619" customWidth="1"/>
-    <col min="15" max="15" width="14" style="2" customWidth="1"/>
-    <col min="16" max="16" width="13.8190476190476" customWidth="1"/>
-    <col min="17" max="17" width="9.18095238095238" style="4"/>
-    <col min="18" max="18" width="9.54285714285714" style="5" customWidth="1"/>
-    <col min="19" max="19" width="13" customWidth="1"/>
-    <col min="20" max="22" width="10" customWidth="1"/>
-    <col min="24" max="24" width="11.8761904761905" customWidth="1"/>
-    <col min="25" max="25" width="9.37142857142857" customWidth="1"/>
+    <col min="3" max="4" width="16" style="2" customWidth="1"/>
+    <col min="5" max="7" width="12.7238095238095" style="2" customWidth="1"/>
+    <col min="8" max="9" width="19.1809523809524" style="2" customWidth="1"/>
+    <col min="10" max="11" width="15.2666666666667" style="2" customWidth="1"/>
+    <col min="12" max="12" width="16" style="2" customWidth="1"/>
+    <col min="13" max="13" width="12.8190476190476" style="2" customWidth="1"/>
+    <col min="14" max="15" width="22.1809523809524" style="3" customWidth="1"/>
+    <col min="16" max="16" width="11.5428571428571" customWidth="1"/>
+    <col min="17" max="17" width="15.447619047619" customWidth="1"/>
+    <col min="18" max="18" width="14" style="2" customWidth="1"/>
+    <col min="19" max="19" width="13.8190476190476" customWidth="1"/>
+    <col min="20" max="20" width="9.18095238095238" style="4"/>
+    <col min="21" max="21" width="9.54285714285714" style="5" customWidth="1"/>
+    <col min="22" max="22" width="13" customWidth="1"/>
+    <col min="23" max="25" width="10" customWidth="1"/>
+    <col min="27" max="27" width="11.8761904761905" customWidth="1"/>
+    <col min="28" max="28" width="9.37142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:28">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1361,58 +1388,58 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="5" t="s">
         <v>20</v>
       </c>
       <c r="V1" s="9" t="s">
@@ -1424,217 +1451,217 @@
       <c r="X1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="11"/>
+      <c r="Y1" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="10"/>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:28">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="3">
+      <c r="G2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="3">
         <v>1</v>
       </c>
-      <c r="L2" s="3">
+      <c r="O2" s="3">
         <v>2</v>
-      </c>
-      <c r="M2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="P2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" s="4">
+      <c r="Q2" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="S2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T2" s="4">
         <v>1</v>
       </c>
-      <c r="R2" s="5">
+      <c r="U2" s="5">
         <v>480000</v>
       </c>
-      <c r="S2">
-        <f>Q2*R2</f>
+      <c r="V2">
+        <f>T2*U2</f>
         <v>480000</v>
       </c>
-      <c r="T2">
+      <c r="W2">
         <v>10</v>
       </c>
-      <c r="U2">
-        <f>S2*(T2/100)</f>
+      <c r="X2">
+        <f>V2*(W2/100)</f>
         <v>48000</v>
       </c>
-      <c r="V2">
+      <c r="Y2">
         <v>1</v>
       </c>
-      <c r="W2">
+      <c r="Z2">
         <v>1</v>
       </c>
-      <c r="X2" s="10">
-        <f>SUM(S2,U2)</f>
+      <c r="AA2" s="11">
+        <f>SUM(V2,X2)</f>
         <v>528000</v>
       </c>
-      <c r="Y2" s="12"/>
+      <c r="AB2" s="12"/>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:27">
       <c r="A3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="P3" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q3" s="4">
+        <v>27</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="S3" t="s">
+        <v>38</v>
+      </c>
+      <c r="T3" s="4">
         <v>2</v>
       </c>
-      <c r="R3" s="5">
+      <c r="U3" s="5">
         <v>1600</v>
       </c>
-      <c r="S3">
-        <f>Q3*R3</f>
+      <c r="V3">
+        <f>T3*U3</f>
         <v>3200</v>
       </c>
-      <c r="T3">
+      <c r="W3">
         <v>10</v>
       </c>
-      <c r="U3">
-        <f>S3*(T3/100)</f>
+      <c r="X3">
+        <f>V3*(W3/100)</f>
         <v>320</v>
       </c>
-      <c r="V3">
+      <c r="Y3">
         <v>1</v>
       </c>
-      <c r="X3" s="10">
-        <f>SUM(S3,U3)</f>
+      <c r="AA3" s="11">
+        <f>SUM(V3,X3)</f>
         <v>3520</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:27">
       <c r="A4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="P4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q4" s="4">
+        <v>27</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>39</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="S4" t="s">
+        <v>41</v>
+      </c>
+      <c r="T4" s="4">
         <v>3</v>
       </c>
-      <c r="R4" s="5">
+      <c r="U4" s="5">
         <v>480000</v>
       </c>
-      <c r="S4">
-        <f>Q4*R4</f>
+      <c r="V4">
+        <f>T4*U4</f>
         <v>1440000</v>
       </c>
-      <c r="T4">
+      <c r="W4">
         <v>10</v>
       </c>
-      <c r="U4">
-        <f>S4*(T4/100)</f>
+      <c r="X4">
+        <f>V4*(W4/100)</f>
         <v>144000</v>
       </c>
-      <c r="V4">
+      <c r="Y4">
         <v>1</v>
       </c>
-      <c r="X4" s="10">
-        <f>SUM(S4,U4)</f>
+      <c r="AA4" s="11">
+        <f>SUM(V4,X4)</f>
         <v>1584000</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:27">
       <c r="A5" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="3">
+      <c r="G5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N5" s="3">
         <v>2</v>
       </c>
-      <c r="L5" s="3">
+      <c r="O5" s="3">
         <v>2</v>
       </c>
-      <c r="M5" t="s">
-        <v>29</v>
-      </c>
-      <c r="N5" t="s">
-        <v>40</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q5" s="4">
+      <c r="P5" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>43</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="T5" s="4">
         <v>3</v>
       </c>
-      <c r="R5" s="5">
+      <c r="U5" s="5">
         <v>230000</v>
       </c>
-      <c r="S5">
-        <f>Q5*R5</f>
+      <c r="V5">
+        <f>T5*U5</f>
         <v>690000</v>
       </c>
-      <c r="U5">
-        <f>S5*(T5/100)</f>
+      <c r="X5">
+        <f>V5*(W5/100)</f>
         <v>0</v>
       </c>
-      <c r="V5">
+      <c r="Y5">
         <v>1</v>
       </c>
-      <c r="W5">
+      <c r="Z5">
         <v>1</v>
       </c>
-      <c r="X5" s="10">
-        <f>SUM(S5,U5)</f>
+      <c r="AA5" s="11">
+        <f>SUM(V5,X5)</f>
         <v>690000</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:27">
       <c r="A6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X6" s="10"/>
-    </row>
-    <row r="7" spans="24:24">
-      <c r="X7" s="10"/>
-    </row>
-    <row r="8" spans="24:24">
-      <c r="X8" s="10"/>
-    </row>
-    <row r="9" spans="24:24">
-      <c r="X9" s="10"/>
+        <v>45</v>
+      </c>
+      <c r="AA6" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1657,53 +1684,53 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update handle paymend method on import invoice excel file
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoice_mtt/MauUploadHDMTT-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoice_mtt/MauUploadHDMTT-TT78.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8940"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,8 @@
 2: Chuyển khoản
 3: Tiền mặt/ chuyển khoản
 4: Đối trừ công nợ
-5: Không thu tiền</t>
+5: Không thu tiền
+6: “” (Không ghi hình thức)</t>
         </r>
       </text>
     </comment>
@@ -518,37 +519,37 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="34">
@@ -1043,7 +1044,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>

</xml_diff>